<commit_message>
Update workouts import message and template instructions
Import now saves every valid row and emails the list of rows that could
not be saved, and duplicates are detected by name and description.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NQ2YuTZnySBnhY6h1d6Vfk
</commit_message>
<xml_diff>
--- a/src/assets/templates/workouts-import-template.xlsx
+++ b/src/assets/templates/workouts-import-template.xlsx
@@ -493,19 +493,14 @@
           <t>Upute za uvoz vježbi</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>Vježbe unosite u prvi list (Vjezbe), jedna vježba po retku, ispod zaglavlja.</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -513,12 +508,8 @@
           <t>Ne mijenjajte nazive stupaca u zaglavlju.</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -539,7 +530,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Naziv vježbe na hrvatskom (obavezno). Vježbe čiji naziv već postoji preskaču se.</t>
+          <t>Naziv vježbe na hrvatskom (obavezno).</t>
         </is>
       </c>
     </row>
@@ -551,7 +542,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Opis vježbe na hrvatskom.</t>
+          <t>Opis vježbe na hrvatskom. Vježbe s istim nazivom i opisom kao postojeće (ili ranije u datoteci) preskaču se kao duplikati.</t>
         </is>
       </c>
     </row>
@@ -580,7 +571,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
@@ -640,7 +630,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
@@ -651,7 +640,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Nazivi i opisi automatski se prevode na engleski i talijanski.</t>
+          <t>Nazivi i opisi automatski se prevode na engleski i talijanski. Uvoz radi u pozadini: sve ispravne vježbe se spremaju, a na email dobivate rezultat, popis vježbi koje nisu spremljene s razlogom te Excel datoteku s tim vježbama koju možete ispraviti i ponovno uvesti.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make workout video optional and add Language column to import template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NQ2YuTZnySBnhY6h1d6Vfk
</commit_message>
<xml_diff>
--- a/src/assets/templates/workouts-import-template.xlsx
+++ b/src/assets/templates/workouts-import-template.xlsx
@@ -438,13 +438,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,6 +467,11 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>WorkoutTypes</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Language</t>
         </is>
       </c>
     </row>
@@ -480,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -530,7 +536,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Naziv vježbe na hrvatskom (obavezno).</t>
+          <t>Naziv vježbe (obavezno), na jeziku iz stupca Language.</t>
         </is>
       </c>
     </row>
@@ -542,7 +548,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Opis vježbe na hrvatskom. Vježbe s istim nazivom i opisom kao postojeće (ili ranije u datoteci) preskaču se kao duplikati.</t>
+          <t>Opis vježbe, na jeziku iz stupca Language. Vježbe s istim nazivom i opisom kao postojeće (ili ranije u datoteci) preskaču se kao duplikati.</t>
         </is>
       </c>
     </row>
@@ -554,7 +560,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>YouTube poveznica videa (obavezno), npr. https://www.youtube.com/watch?v=IODxDxX7oi4</t>
+          <t>YouTube poveznica videa (neobavezno, može se dodati kasnije), npr. https://www.youtube.com/watch?v=IODxDxX7oi4</t>
         </is>
       </c>
     </row>
@@ -571,76 +577,100 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="4" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Jezik teksta u retku: HR, EN ili IT (neobavezno, prazno = HR).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Primjer retka</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Čučanj</t>
-        </is>
-      </c>
+      <c r="B13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Osnovna vježba za noge i stražnjicu.</t>
+          <t>Čučanj</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>VideoUrl</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=aclHkVaku9U</t>
+          <t>Osnovna vježba za noge i stražnjicu.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>VideoUrl</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=aclHkVaku9U</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>WorkoutTypes</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Snaga, Noge</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Napomena</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Nazivi i opisi automatski se prevode na engleski i talijanski. Uvoz radi u pozadini: sve ispravne vježbe se spremaju, a na email dobivate rezultat, popis vježbi koje nisu spremljene s razlogom te Excel datoteku s tim vježbama koju možete ispraviti i ponovno uvesti.</t>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Nazivi, opisi i nove vrste vježbi automatski se prevode s jezika retka na ostale jezike (HR, EN, IT). Uvoz radi u pozadini: sve ispravne vježbe se spremaju, a na email dobivate rezultat, popis vježbi koje nisu spremljene s razlogom te Excel datoteku s tim vježbama koju možete ispraviti i ponovno uvesti.</t>
         </is>
       </c>
     </row>

</xml_diff>